<commit_message>
updated scraper with new keywords
</commit_message>
<xml_diff>
--- a/efe_mena_education_grants.xlsx
+++ b/efe_mena_education_grants.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -545,471 +545,1255 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>UNHCR seeks Monitoring, Evaluation, and Learning (MEL) specialists, academic centers, and NGOs to design and implement a comprehensive MEL system for its Educate a Child program. This initiative, operating across Chad, Kenya, Pakistan, Uganda, and Syria, focuses on strengthening refugee learning systems, developing data dashboards, and facilitating regional synthesis to improve education access for displaced children.</t>
+          <t>UNHCR is seeking MEL specialists, academic centers, and NGOs to design and implement a comprehensive Monitoring, Evaluation, and Learning system for its Educate a Child (EAC) program. This initiative supports refugee learning systems, data dashboards, and regional synthesis, aiming to improve education access for displaced children across Chad, Kenya, Pakistan, Uganda, and Syria.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="80" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-a9f</t>
+          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-f41</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Minority Rights Group</t>
+          <t>Sharjah Entrepreneurship Center</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>EUR €20,000; one grant per country; duration up to 12 months.</t>
+          <t>Pilot funding of AED 250,000.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Lebanon, Tunisia, Palestine, Morocco.</t>
+          <t>Pilots must be implemented in the UAE (Sharjah),</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Human Rights; Focus areas: minority-led networks, policy change, MENA.</t>
+          <t>Education, early childhood, innovation.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Human rights CSOs coordinating or forming issue-based networks in listed countries.</t>
+          <t>Startups from anywhere in the world, ready for scaling, ideally at Series A or B funding stages with an adequate team size.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://minorityrights.org/jobs/macs-networks/</t>
+          <t>https://www.asc.sheraa.ae/</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>December 21, 2025.</t>
+          <t>August 17, 2025.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>As part of the MACS (Minorities, Accountability and Civic Space) program, this call supports CSOs to build or expand issue-based networks that influence policy change. Grants will fund the creation of physical or digital platforms for collaboration, support umbrella organizations that coordinate advocacy, and enable structured dialogue and campaigning on minority and human rights issues at national or regional levels.</t>
+          <t>The Access Sharjah Challenge (ASC) invites global bold education startups to collaborate in shaping solutions for high-impact, real-world challenges within Sharjah’s two priority sectors: future-ready skills challenge and Arabic in early childhood challenge.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Human rights CSOs coordinating or forming issue-based networks in Lebanon, Tunisia, Palestine, and Morocco can apply for €20,000 grants from Minority Rights Group. This opportunity funds the development or expansion of networks to influence policy change on minority and human rights issues within the MENA region. Grants support collaborative platforms, advocacy coordination, and campaigning efforts for up to 12 months.</t>
+          <t>The Sharjah Entrepreneurship Center's "Education Challenges" grant invites global startups, ideally at Series A/B, to develop innovative solutions in education focusing on future-ready skills and Arabic in early childhood. Selected pilots, which must be implemented in Sharjah, UAE, will receive AED 250,000 in funding.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-870</t>
+          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-f41</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>UN Women Arab States</t>
+          <t>Italian Agency for Development Cooperation (AICS)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>MAD 1,000,000 to 1,250,000</t>
+          <t>EUR €1.4M total; sub-grants of €20,000 – €45,000 (MSMEs/cooperatives), €10,000 – €25,000 (CBOs).</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Morocco (national level)</t>
+          <t>Lebanon.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Gender Norms Transformation; Youth Engagement; Human Rights; supports SDG 5 (Gender Equality), SDG 16 (Peace &amp; Justice)</t>
+          <t>Economic Development; Social Protection; Livelihoods; SDGs 1, 5, 8, 10, 13.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>National Moroccan human rights CSOs with demonstrated experience in youth mobilization and gender rights</t>
+          <t>NGOs legally registered in Lebanon or eligible EU or partner countries; lead applicants must demonstrate prior experience managing sub‑grant schemes, working with SDCs, and driving local economic development. Co‑applicants must meet similar criteria.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://arabstates.unwomen.org/en/programme-implementation/2025/07/call-for-proposals-recruitement-of-a-national-human-rights-cso-to-transform-patriarchal-masculinities-in-youth</t>
+          <t>https://aics.portaleamministrazionetrasparente.it/archivio97_concessione-contributi_0_178_952_1.html</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>September 12, 2025.</t>
+          <t>August 25, 2025 (23:59 Lebanon Time).</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>UN Women Morocco is recruiting a national human rights organization to lead a youth-centered initiative to transform patriarchal masculinities and shift harmful gender norms. The program focuses on empowering young people—especially boys and men—through peer-led advocacy, arts, storytelling, and local campaigns. This national-level initiative is part of the regionalDare to Carestrategy and emphasizes long-term behavior change, community mobilization, and gender rights integration.</t>
+          <t>As part of the EU‑funded ELISSA initiative, AICS is seeking NGOs to lead participatory local economic development programs in Lebanese communities affected by the Syrian crisis. The fund will support capacity-building for Ministry‑recognized Social Development Centers (SDCs) and provide sub‑grants to local operators and CBOs to pilot inclusive, green livelihood initiatives.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>UN Women Morocco invites national Moroccan human rights CSOs with expertise in youth mobilization and gender rights to lead initiatives across Morocco. This funding supports programs focused on transforming patriarchal masculinities and harmful gender norms through peer-led advocacy, arts, and local campaigns. The grant, up to MAD 1,250,000, aims to empower young people to drive long-term behavior change for gender equality.</t>
+          <t>The Italian Agency for Development Cooperation (AICS) invites NGOs registered in Lebanon, eligible EU, or partner countries with experience in sub-grant management and local economic development to apply for its Local Economic Development Grant Program in Lebanon. This initiative, part of the EU-funded ELISSA program, seeks proposals to lead participatory local economic development in Lebanese communities affected by the Syrian crisis, funding capacity-building for Social Development Centers and providing sub-grants for inclusive, green livelihood initiatives by MSMEs, cooperatives, and CBOs.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-870</t>
+          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-b0a</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>European Commission</t>
+          <t>The Digital Defenders Partnership (DDP).</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Total envelope available is EUR €10.2M, they expect to award three grants of up to EUR €3.4M</t>
+          <t>Grants of up to EUR €15,000 for projects lasting 6 to 12 months.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Europe and Horizon associated countries (Albania, Armenia, Bosnia and Herzegovina, Canada, Faroe Islands, Georgia, Iceland, Israel, Kosovo, Moldova, Montenegro, New Zealand, North Macedonia, Norway, Serbia, Tunisia, Türkiye, Ukraine, United Kingdom).</t>
+          <t>Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia, and Yemen.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Inclusion, persons with disabilities, human rights, equality.</t>
+          <t>Human rights.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Any legal entity registered in a eligible country.</t>
+          <t>Human rights organizations and collectives</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL2-2025-01-TRANSFO-09?isExactMatch=true&amp;status=31094501,31094502&amp;order=DESC&amp;pageNumber=3&amp;pageSize=50&amp;sortBy=startDate</t>
+          <t>https://apply.grants.digitaldefenders.org/</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>September 16, 2025.</t>
+          <t>May 7, 2025.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Projects should contribute to some of the following expected outcomes (minimum three outcomes); 1. Develop innovative evidence-based policy approaches to promote the autonomy of persons with disabilities of any age and any origin of the disability or impairment; 2. Develop practices that facilitate the full inclusion and participation of persons with disabilities in different areas of life, including education, family life, employment, living arrangements, leisure, arts, culture and sport on equal basis with others; 3. Address the seamless use of accessible and assistive technology, including digital technologies and artificial intelligence, in the community and related services and infrastructure. If possible, identify specific measures and tools for different addressed areas of lives of persons with disabilities, such as education, recruitment, hiring, return to work, and independent life; 4. Identify and compare the usefulness of different options for policies and measures aiming to increase the autonomy and quality of life of persons with disabilities, as well as the quality of life and well-being of their families, using a person-centered approach, taking into account the individual needs of persons with disabilities and ensuring their full enjoyment of human rights and fundamental freedoms on equal basis with others; 5. Identify relevant actors to achieve effective results (public actors, civil society organizations, private sector, social economy actors, etc.) and explore their roles and interaction, with a view to assessing integration among different social, support and essential services (including e.g. transport or housing) necessary to promote autonomy and inclusion in the community.</t>
+          <t>Invites human rights organizations and collectives from the SWANA region (Southwest Asia and North Africa) to apply for the Sustainable Protection Fund. This fund supports long-term digital security capacity building. The fund prioritizes organizations and collectives working on: Media and freedom of expression, Civil and political rights, Feminist and LGBTQ+ movements.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>The European Commission invites legal entities registered in Europe and Horizon associated countries to apply for grants supporting the increased autonomy and full inclusion of persons with disabilities. Projects should develop innovative, evidence-based policy approaches and practices, including accessible and assistive technology, to facilitate full inclusion and participation across various life areas. The goal is to identify person-centered solutions that enhance the quality of life and ensure the full enjoyment of human rights for persons with disabilities.</t>
+          <t>The Digital Defenders Partnership invites human rights organizations and collectives from Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia, and Yemen to apply for the Sustainable Protection Fund. This fund offers grants up to EUR €15,000 for 6-12 month projects focused on long-term digital security capacity building. Priority is given to initiatives promoting media/freedom of expression, civil/political rights, and feminist/LGBTQ+ movements.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-870</t>
+          <t>https://impactfunding.substack.com/p/agriculture-climate-environment-energy-c1f</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>European Commission</t>
+          <t>Conservation Leadership Programme (CLP)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Total envelope available is EUR €10.2M, they expect to award three grants of up to EUR €3.4M</t>
+          <t>Up to USD $15,000 per team; CLP must cover at least 50% of the total budget.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Europe and Horizon associated countries (Albania, Armenia, Bosnia and Herzegovina, Canada, Faroe Islands, Georgia, Iceland, Israel, Kosovo, Moldova, Montenegro, New Zealand, North Macedonia, Norway, Serbia, Tunisia, Türkiye, Ukraine, United Kingdom).</t>
+          <t>LMICs in Africa, Asia, Latin America &amp; Caribbean, Pacific, Eastern &amp; Southeastern Europe, and Middle East.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Education, EdTech, children’s well-being.</t>
+          <t>Biodiversity &amp; Ecosystems; Focus areas: threatened species, habitat management, youth capacity building, field-based conservation.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Any legal entity registered in a eligible country.</t>
+          <t>Teams of at least three nationals of the project country; all must be early-career conservationists with &lt;5 years’ experience.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://grants.fundsforngospremium.com/opportunity/op/cfps-impact-of-the-learning-environment-and-the-use-of-digital-tools-programme</t>
+          <t>https://www.conservationleadershipprogramme.org/awards-opportunities/team-awards/future-conservationist-award/</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>September 16, 2025.</t>
+          <t>January 9, 2026 (11:59 p.m. GMT).</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Digital devices and tools are an integral part in the lives of children and teenagers as they grow. There is discussion about the impact of the use of digital tools in everyday life on children’s wellbeing (cognitive, emotional, social) and development, but the evidence is often piecemeal. Proposals should investigate the impact that the expansion and normalization of children’s use of digital technologies (including generative AI) in everyday life has on their learning, at a time in their lives when literacy and numeracy skills are developing, and during adolescence. Projects should contribute to all of the following expected outcomes: 1. Provide analyses of the impact of digital tools in everyday life on wellbeing and how children learn. 2. Provide analyses and evidence-based recommendations on how to provide opportunities for high quality education that uses digital technologies in ways that support the wellbeing of the school community (students, teachers and school leaders).</t>
+          <t>This prestigious early-career award supports emerging conservationists to lead field-based projects that protect threatened species and habitats across the Global South. With a strong emphasis on leadership development, grantees receive funding, mentorship, and access to a global alumni network. Proposed projects must be focused on protecting species categorized by the IUCN Red List as globally threatened (Critically Endangered, Endangered, Vulnerable) or Data Deficient, or when there is information indicating the need for urgent conservation action. Projects may address themes such as climate impact and adaptation, habitat restoration and/or management, social development and wellbeing, Indigenous community participation, and/or environmental policy. Projects must also address urgent ecological threats while promoting inclusive community engagement and the application of conservation science. The initiative prioritizes diversity, local ownership, and measurable on-the-ground outcomes, offering an essential launchpad for young professionals in the biodiversity space.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>The European Commission invites legal entities registered in Europe and Horizon associated countries to apply for grants up to €3.4M to research the impact of digital tools and the learning environment on children's key skills, competence development, and wellbeing. Projects should analyze the effect of digital technologies, including generative AI, on children's learning and provide evidence-based recommendations for high-quality, supportive EdTech in education.</t>
+          <t>The Conservation Leadership Programme (CLP) offers its Future Conservationist Award, providing up to $15,000 to early-career teams (less than five years' experience) who are nationals of the project country in LMICs across Africa, Asia, Latin America &amp; Caribbean, Pacific, Eastern &amp; Southeastern Europe, and the Middle East. This grant supports field-based conservation projects that protect threatened species and habitats, while also fostering leadership development and inclusive community engagement.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-f41</t>
+          <t>https://impactfunding.substack.com/p/agriculture-climate-environment-energy-323</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Sharjah Entrepreneurship Center</t>
+          <t>Biodiversa+</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Pilot funding of AED 250,000.</t>
+          <t>Approx. EUR €40 million total to be allocated across consortia.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Pilots must be implemented in the UAE (Sharjah),</t>
+          <t>Belgium, Brazil, Bulgaria, Czech Republic, Denmark, Estonia, Faroe Islands, France, Ireland, Iceland, Italy, Israel, South Africa, Latvia, Lithuania, Hungary, Moldova, Germany, Netherlands, Norway, Poland, Portugal, Austria, Romania, Slovakia, Slovenia, Spain, Sweden, Switzerland, Taiwan, Tunisia, Turkey.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Education, early childhood, innovation.</t>
+          <t>biodiversity conservation, sustainability science, policy engagement, community-led research / SDG 15, SDG 17.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Startups from anywhere in the world, ready for scaling, ideally at Series A or B funding stages with an adequate team size.</t>
+          <t>International consortia of at least three partners from participating countries, including minimum two EU Member or Associated States.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://www.asc.sheraa.ae/</t>
+          <t>https://www.biodiversa.eu/research-funding/upcoming-calls/</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>August 17, 2025.</t>
+          <t>Pre‑proposals due early November 7, 2025 ; full proposals due early April 2026.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>The Access Sharjah Challenge (ASC) invites global bold education startups to collaborate in shaping solutions for high-impact, real-world challenges within Sharjah’s two priority sectors: future-ready skills challenge and Arabic in early childhood challenge.</t>
+          <t>This transnational transnational call will fund interdisciplinary research consortia working to restore ecosystem integrity and connectivity. Projects must address long-term sustainability, measurable ecological success, and transdisciplinary integration of ecological, socio-economic, and cultural dimensions. Proposals should support global biodiversity frameworks and explore future-proof restoration strategies including predictive modelling and novel methods.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>The Sharjah Entrepreneurship Center invites global Series A or B education startups to propose scalable solutions for real-world challenges. This opportunity offers AED 250,000 in pilot funding for projects implemented in Sharjah, UAE, addressing future-ready skills or Arabic in early childhood.</t>
+          <t>Biodiversa+ invites international consortia of at least three partners from participating countries (minimum two EU Member or Associated States) to apply for funding. The "BiodivConnect Call" supports interdisciplinary research projects focused on restoring ecosystem functioning, integrity, and connectivity, emphasizing long-term sustainability, transdisciplinary integration, and future-proof strategies within biodiversity conservation and sustainability science across Europe, South America, Africa, and Asia.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-f41</t>
+          <t>https://impactfunding.substack.com/p/agriculture-climate-environment-energy-e29</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Italian Agency for Development Cooperation (AICS)</t>
+          <t>European Commission</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>EUR €1.4M total; sub-grants of €20,000 – €45,000 (MSMEs/cooperatives), €10,000 – €25,000 (CBOs).</t>
+          <t>Grants of €1,000–€50,000 per MSME; up to €50,000 per city; total budget €250,000.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Lebanon.</t>
+          <t>Kenya; Uganda; South Africa; Burkina Faso; Tunisia.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Economic Development; Social Protection; Livelihoods; SDGs 1, 5, 8, 10, 13.</t>
+          <t>Circular Food Systems; Urban Food Security.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>NGOs legally registered in Lebanon or eligible EU or partner countries; lead applicants must demonstrate prior experience managing sub‑grant schemes, working with SDCs, and driving local economic development. Co‑applicants must meet similar criteria.</t>
+          <t>Circular food MSMEs with 1–50 staff and ≤ €50K revenue, operating in designated hub city, having completed local incubator training; no owner employed by government.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://aics.portaleamministrazionetrasparente.it/archivio97_concessione-contributi_0_178_952_1.html</t>
+          <t>https://afrifoodlinks.org/grants-for-food-smes/</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>August 25, 2025 (23:59 Lebanon Time).</t>
+          <t>September 17, 2025 (23:59 CET).</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>As part of the EU‑funded ELISSA initiative, AICS is seeking NGOs to lead participatory local economic development programs in Lebanese communities affected by the Syrian crisis. The fund will support capacity-building for Ministry‑recognized Social Development Centers (SDCs) and provide sub‑grants to local operators and CBOs to pilot inclusive, green livelihood initiatives.</t>
+          <t>This cascade grant under the EU AfriFOODlinks project supports circular (food) MSMEs in five cities (Kisumu, Mbale, Cape Town, Ouagadougou, Tunis)that have completed local AfriFOODlinks incubation. Businesses with 1–50 employees and ≤ €50,000 in revenue can receive €1,000–€50,000 to boost circularity, internal systems, and readiness for market growth. Priority goes to youth- and women-led ventures; mandatory language requirements apply based on city.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>The Italian Agency for Development Cooperation (AICS) offers funding to NGOs legally registered in Lebanon or eligible EU/partner countries, especially those experienced in sub-grant management and local economic development. This program aims to foster participatory local economic development in Lebanese communities impacted by the Syrian crisis by strengthening Social Development Centers and providing sub-grants for inclusive, green livelihood initiatives.</t>
+          <t>The European Commission invites circular food MSMEs (1-50 staff, ≤€50K revenue) that have completed AfriFOODlinks incubation and operate in designated hub cities across Kenya, Uganda, South Africa, Burkina Faso, and Tunisia to apply. Grants from €1,000 to €50,000 are available to enhance their circularity, strengthen internal systems, and prepare for market growth within urban food security, with priority for youth- and women-led ventures.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-b0a</t>
+          <t>https://impactfunding.substack.com/p/gender-equality-and-women-empowerment-6e5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Minority Rights Group</t>
+          <t>inDrive</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Grants range EUR €11,000 - €33,000.</t>
+          <t>USD $100,000 total pool; Top3 awards: $50,000 (1st), $30,000 (2nd), $20,000 (3rd).</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lebanon, Tunisia, Morocco and Palestine.</t>
+          <t>Global, with emphasis on emerging markets (Africa, Latin America, Asia, MENA).</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Migrants, inclusion, advocacy.</t>
+          <t>Technology; Focus areas: women tech founders, early‑stage startups, global scaling.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>human rights and minority rights/ minority groups led nonprofit organizations</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+          <t>Start‑ups founded or co‑founded and led by a woman; ≤5 years old; functional prototype; ≤USD 6 m total funding; must present in English.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.auroratechaward.com/</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>May 4, 2025.</t>
+          <t>November 12, 2025 (23:59 UTC).</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Now accepting applications for advocacy grants and core funding grants. These grants are available for Human Rights Civil Society Organizations (CSOs) aim to maximize the attention toward the situation of minorities and marginalized communities in the target countries, and that want to invest in their organizational development, organizational infrastructures or to effectively develop their institutional capacity.</t>
+          <t>This award seeks to identify and uplift high‑potential women‑led tech startups from emerging markets, providing not just capital but strategic visibility, mentorship and access to a global investor network. By focusing on founders who are less than 5 years into their venture, have developed a functional prototype and have raised under USD 6 million in total funding, the program aims to correct the systemic gender funding gap and accelerate scaling of startups that might otherwise be overlooked.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Minority Rights Group offers advocacy and core funding grants for human rights and minority-led non-profit Civil Society Organizations (CSOs) in Lebanon, Tunisia, Morocco, and Palestine. These grants support efforts to highlight the situation of minorities and marginalized communities, alongside investments in organizational development, infrastructure, and institutional capacity.</t>
+          <t>The Aurora Tech Award, sponsored by inDrive, offers $100,000 in prizes to early-stage technology startups, less than five years old with a functional prototype, that are founded or co-founded and led by a woman. This global opportunity specifically targets high-potential women-led tech ventures in emerging markets across Africa, Latin America, Asia, and MENA, aiming to accelerate their growth and global scaling.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-b0a</t>
+          <t>https://impactfunding.substack.com/p/gender-equality-and-women-empowerment-6d7</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The Digital Defenders Partnership (DDP).</t>
+          <t>Women’s Peace and Humanitarian Fund (WPHF)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Grants of up to EUR €15,000 for projects lasting 6 to 12 months.</t>
+          <t>Grants range USD $2,500 – $30,000 (institutional), and USD $30,000 – $200,000 (programmatic).</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia, and Yemen.</t>
+          <t>Syria.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Human rights.</t>
+          <t>Humanitarian Assistance; Focus areas: displacement, economic empowerment, mental health, civic participation, justice access.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Human rights organizations and collectives</t>
+          <t>Legally registered Syrian CSOs led by women, young women, or displaced individuals; youth-focused and feminist organizations.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://apply.grants.digitaldefenders.org/</t>
+          <t>https://wphfund.org/call-for-proposals-in-syria-2/</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>May 7, 2025.</t>
+          <t>October 20, 2025 (11:59pm Geneva Time).</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Invites human rights organizations and collectives from the SWANA region (Southwest Asia and North Africa) to apply for the Sustainable Protection Fund. This fund supports long-term digital security capacity building. The fund prioritizes organizations and collectives working on: Media and freedom of expression, Civil and political rights, Feminist and LGBTQ+ movements.</t>
+          <t>In a rapidly deteriorating humanitarian landscape, WPHF is calling on Syrian women- and youth-led civil society organizations to step into leadership roles across peacebuilding, response, and recovery. This fund supports both institutional development and programmatic work aligned with three core Impact Areas: humanitarian response, protection and mental health, and peacebuilding for displaced women. The call reflects WPHF’s investment in feminist crisis leadership, intersectional justice, and inclusive systems transformation — with particular attention to displaced, disabled, and marginalized groups. Projects must be rooted in community realities and prioritize long-term sustainability, feminist M&amp;E, and collaborative delivery.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>The Digital Defenders Partnership's Sustainable Protection Fund invites human rights organizations and collectives across Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia, and Yemen to apply. This fund offers grants of up to EUR €15,000 for 6-12 month projects focused on long-term digital security capacity building, prioritizing initiatives supporting media freedom, civil rights, and feminist/LGBTQ+ movements.</t>
+          <t>The Women's Peace and Humanitarian Fund (WPHF) is inviting proposals from legally registered Syrian CSOs led by women, young women, or displaced individuals, including youth-focused and feminist organizations, to address the humanitarian crisis in Syria. This funding supports both institutional development and programmatic work in humanitarian response, protection and mental health, and peacebuilding for displaced women, with a focus on areas like displacement, economic empowerment, civic participation, and justice access. Grants range from $2,500 to $200,000 depending on the project type.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>https://impactfunding.substack.com/p/education-human-rights-and-inclusion-b0a</t>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-emergency-programming-30d</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>The Digital Defenders Partnership (DDP).</t>
+          <t>ActionAid</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Grants of up to EUR €25,000 for a period of up to 1 year.</t>
+          <t>Grant size equivalent to GBP £100,000 per grant.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia, and Yemen.</t>
+          <t>Syria.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Internet freedom, human rights.</t>
+          <t>Humanitarian Response; Focus areas: women-led protection, youth-led recovery, community resilience.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Human rights organizations and collectives</t>
+          <t>Syrian local and national civil society organizations, with priority to women- and youth-led groups.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://apply.grants.digitaldefenders.org/</t>
+          <t>https://reliefweb.int/job/4195140/call-proposal-cfp-syria-turkiye-earthquake-emergency-response-2025-actionaid-arab-region-aaar</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>May 7, 2025.</t>
+          <t>February 8, 2026 (23:59 Jordan/Syria Time).</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Through this fund, DDP provides to support organizations and collectives working to advance internet freedom and protect human rights defenders (HRDs) from a holistic perspective. They welcome a wide range of initiatives that strengthen digital rights and support HRDs at risk. Funded activities may include (but are not limited to): Ensuring internet access during shutdowns, slowdowns, censorship, or infrastructure disruption, Providing digital security training, accompaniment, or broader protection support to HRDs, Offering technical expertise such as digital forensic analysis, secure hosting, or other vital services for civil society, Engaging in advocacy and lobbying efforts to defend digital rights and online freedom, Covering core costs for high-impact organizations or collectives with limited access to other funding.</t>
+          <t>Through this call, ActionAid Arab Region seeks to advance a locally led transition from emergency response to early recovery for communities in Syria affected by the 2023 earthquake, protracted conflict, and evolving return dynamics. The funding is explicitly framed around shifting power to women- and youth-led local organizations, positioning them not only as implementers but as leaders shaping protection, recovery, and resilience strategies in volatile contexts. Priority is given to interventions that integrate protection, livelihoods, community cohesion, and advocacy, while responding to the specific risks faced by returnees, internally displaced people, and host communities. By combining humanitarian action with early recovery and policy influence, the call reflects ActionAid’s commitment to localization, gender justice, and youth leadership as central drivers of sustainable recovery in crisis-affected settings.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>The Digital Defenders Partnership (DDP) invites human rights organizations and collectives in the SWANA region (Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia, and Yemen) to apply for grants up to €25,000. This fund supports initiatives advancing internet freedom and protecting human rights defenders, covering activities such as ensuring internet access, digital security training, technical expertise, advocacy, and organizational core costs.</t>
+          <t>ActionAid offers £100,000 grants to Syrian local and national civil society organizations, prioritizing women- and youth-led groups, for emergency response and early recovery initiatives across Syria. This funding supports projects focused on women-led protection, youth-led recovery, and community resilience for communities affected by the 2023 earthquake, protracted conflict, and evolving return dynamics. Interventions should integrate protection, livelihoods, community cohesion, and advocacy, particularly for returnees, internally displaced people, and host communities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-emergency-programming-6ee</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Innovative Private Sector Development II (IPSD II)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Up to USD 50,000 (Pre‑Investment Grant); up to USD 350,000 (Co‑Investment Grant).</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>West Bank, Palestine.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Economic Development; Focus areas: investment readiness, private capital attraction, business model strengthening.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Tech‑enabled startups and innovative SMEs legally registered or committed to register in the West Bank, operational ≥3 months with revenues ≤ USD 5M.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://ipsd.ps/content/programs/ignite-program.html?utm_source=chatgpt.com</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>January 14, 2026 .</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>This flagship investment readiness program under IPSD II supports tech‑enabled startups and innovative small and medium enterprises in the West Bank by strengthening their capacity to engage investors and scale. The program combines structured business readiness training, one‑on‑one coaching, and facilitated investor engagement to help entrepreneurs refine business models, navigate investor expectations, and prepare compelling investment packages. Eligible firms may also apply for Pre‑Investment Grants of up to USD 50,000 to address commercialization gaps and improve their attractiveness to private capital, with further pathways to larger Co‑Investment Grants (up to USD 350,000) once investment traction is demonstrated. The process includes an initial selection and onboarding phase designed to ensure participants are well positioned for meaningful capital‑raising outcomes.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>This flagship investment readiness program under IPSD II supports tech‑enabled startups and innovative small and medium enterprises in the West Bank by strengthening their capacity to engage investors and scale. The program combines structured business readiness training, one‑on‑one coaching, and facilitated investor engagement to help entrepreneurs refine business models, navigate investor expectations, and prepare compelling investment packages. Eligible firms may also apply for Pre‑Investment Grants of up to USD 50,000 to address commercialization gaps and improve their attractiveness to private capital, with further pathways to larger Co‑Investment Grants (up to USD 350,000) once investment traction is demonstrated. The process includes an initial selection and onboarding phase designed to ensure participants are well positioned for meaningful capital‑raising outcomes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-emergency-programming-6ee</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>UNICEF</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Approx. ILS ₪5,000,000 per partner (12-month project budget).</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Gaza Strip, State of Palestine.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Protection; Focus areas: child protection, psychosocial support, legal assistance, family strengthening.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Registered national or international NGOs and CSOs active in Gaza and enrolled in the UN Partner Portal.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.unpartnerportal.org/cfei/open/18314</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>January 15, 2026.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>This Expression of Interest invites NGOs and CSOs to partner with UNICEF in delivering emergency child protection and MHPSS services while strengthening inclusive justice systems in Gaza. The initiative supports UNICEF’s 2023–2027 programme, aligned with national frameworks and humanitarian coordination. Priorities include case management, psychosocial support, legal aid, kinship care, disability-inclusive services, and outreach around child rights and UXO risks. Prospective partners must demonstrate operational capacity, engage in CP-AoR structures, and align activities with national protection referral pathways. Funding is allocated based on programmatic alignment and cost-effectiveness, with a focus on high-vulnerability areas.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>This Expression of Interest invites NGOs and CSOs to partner with UNICEF in delivering emergency child protection and MHPSS services while strengthening inclusive justice systems in Gaza. The initiative supports UNICEF’s 2023–2027 programme, aligned with national frameworks and humanitarian coordination. Priorities include case management, psychosocial support, legal aid, kinship care, disability-inclusive services, and outreach around child rights and UXO risks. Prospective partners must demonstrate operational capacity, engage in CP-AoR structures, and align activities with national protection referral pathways. Funding is allocated based on programmatic alignment and cost-effectiveness, with a focus on high-vulnerability areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-emergency-programming-cc2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Flat6Labs</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Funding not specified. Access to training, mentorship, and Flat6Labs networks.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Palestine.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Entrepreneurship &amp; MSME Support; Focus areas: business modeling, pre-acceleration, validation, startups.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Palestine-based early-stage startups across sectors.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://flat6labs.com/program/nawah-pre-accelerator-program/</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>September 14, 2025</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Flat6Labs is opening applications for the Palestine edition of the Nawah Pre-Accelerator—a 4-week in-person program in Ramallah designed to help early-stage Palestinian startups validate their ideas and prepare for investment. Through tailored workshops, expert mentorship, and peer collaboration, participants will refine their business models and build traction strategies. The program serves as a launchpad for founders seeking to scale, pitch to investors, and join Flat6Labs’ broader venture-building network.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Flat6Labs is opening applications for the Palestine edition of the Nawah Pre-Accelerator—a 4-week in-person program in Ramallah designed to help early-stage Palestinian startups validate their ideas and prepare for investment. Through tailored workshops, expert mentorship, and peer collaboration, participants will refine their business models and build traction strategies. The program serves as a launchpad for founders seeking to scale, pitch to investors, and join Flat6Labs’ broader venture-building network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-emergency-programming-cc2</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Italian Agency for Development Cooperation (AICS) – Amman Office</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Up to EUR €1.2M per single entity or EUR €1.8M for joint proposals; total call budget approx. EUR €1.3M.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Jordan, Iraq.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Multi-sector humanitarian assistance (food, health, WASH, education, livelihoods, protection, shelter); humanitarian demining.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>NGOs/CSOs either listed under Italian Law 125/2014 or partnering with a registered Italian entity; must demonstrate humanitarian experience; demining-related applicants need proven technical capacity for survey activities.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://aics.portaleamministrazionetrasparente.it/archivio97_concessione-contributi_0_176_952_1.html</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>September 15, 2025 (15:00 Amman time).</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>AICS Amman has launched a new call inviting NGOs and CSOs registered in Italy or eligible partner countries to implement emergency response and early recovery (LRRD) programming in Jordan and Iraq. The initiative supports two lots: Lot 1, covering protection, health, food security, shelter, WASH, livelihoods, education; and Lot 2, focused on humanitarian demining. Total funding amounts reach up to €1.3 million, with individual project caps of €1.2M (single entity) or €1.8M (joint applications).</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>AICS Amman has launched a new call inviting NGOs and CSOs registered in Italy or eligible partner countries to implement emergency response and early recovery (LRRD) programming in Jordan and Iraq. The initiative supports two lots: Lot 1, covering protection, health, food security, shelter, WASH, livelihoods, education; and Lot 2, focused on humanitarian demining. Total funding amounts reach up to €1.3 million, with individual project caps of €1.2M (single entity) or €1.8M (joint applications).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-and-emergency-programming-b9f</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Humanitarian Innovation Accelerator</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Equity-free funding of up to USD $150,000.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Priority countries include; Afghanistan, Burkina Faso, Chad, Central African Republic, Democratic Republic of Congo, Ethiopia, Haiti, Iraq, Laos, Lebanon, Libya, Mali, Mozambique, Myanmar Niger, Palestine, Somalia, South Sudan, Syria, Ukraine and Yemen. *Applications outside these regions will still be considered if they demonstrate alignment with the call for applications and eligibility criteria.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Multisector, emergency and disaster response.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Established startups, companies, NGOs, and organizations ready to scale impactful solutions with an established presence in the country of implementation.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://innovation.wfp.org/HIAP</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>April 20, 2025.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>The second edition of the HIA aims to support technology-powered solutions addressing pressing challenges faced by vulnerable populations and humanitarian actors. The platform supports selected ventures and solution providers with financial, technical, and methodological support from the WFP Innovation Accelerator and its partner ecosystem. Proposed solutions should work to bridge information gaps, enable financial inclusion, strengthen essential infrastructure, and/ or enhance humanitarian response through data and technology.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>The Humanitarian Innovation Accelerator offers equity-free funding up to $150,000 and expert support to established startups, companies, NGOs, and organizations for technology-powered, multisector solutions that address urgent challenges faced by vulnerable populations and humanitarian actors, focusing on areas like information gaps, financial inclusion, and infrastructure. While prioritizing projects in countries such as Afghanistan, DRC, Ukraine, and Yemen, applications from other regions are also considered if they demonstrate an established presence in their country of implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/humanitarian-aid-and-emergency-programming</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Mercy Corps Ventures.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Equity-free grants of up to $100,000.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Africa, South and Southeast Asia, Latin America, the Caribbean, the Middle East, Pacific Islands, and Western Balkans.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Humanitarian response, climate, vulnerable communities, innovation, crypto.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Startups, NGOs, and more.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://medium.com/mercy-corps-social-venture-fund/anticipatory-action-accelerator-expanding-the-innovation-frontier-for-humanitarian-aid-026319f845c0</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>February 14, 2025.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>This initiative seeks to usher in a new era of humanitarian aid, leveraging innovations in tech such as climate data analytics, AI/ML, and crypto payment rails. The Anticipatory Action Accelerator is focused on the intersection of advanced climate analytics, crypto payments, and humanitarian aid. With selected partners, they aim to push the boundaries to improve the lives and livelihoods of underserved users across the Global South.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Mercy Corps Ventures' Anticipatory Action Accelerator offers equity-free grants up to $100,000 for startups and NGOs innovating at the intersection of advanced climate analytics, crypto payments, and humanitarian aid. This initiative seeks to improve the lives and livelihoods of underserved communities primarily across the Global South, including Africa, South and Southeast Asia, Latin America, the Caribbean, and the Middle East.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/cross-cutting-intersectional-impact-bc1</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Embassy of Japan in Jordan</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>JPY 10,000,000–20,000,000 per project (approx USD $65,000–130,000 / JOD 45,000–90,000).</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Jordan (national).</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Community Development; Focus areas: grassroots human security, socio-economic development, small-scale infrastructure.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>NGOs, municipalities, educational institutions, or health institutions legally registered in Jordan with at least 2 years of operational experience.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.jordan.emb-japan.go.jp/itpr_en/11_000001_01396.html</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>February 7, 2026 .</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>The Grant Assistance for Grassroots Human Security Projects (GGP) is part of Japan’s Official Development Assistance (ODA) framework, designed to support small-scale, community-focused initiatives that directly improve socio-economic conditions at the grassroots level in Jordan. Through this program, the Embassy of Japan seeks projects that deliver tangible benefits, from essential equipment procurement to community infrastructure renovations, supporting locally defined priorities and sustainable development outcomes. The funding logic emphasizes practical, operational impact and community ownership, prioritizing organizations with strong ties to their communities and demonstrated project delivery capacity. A comprehensive application, including financial audits, price quotations, feasibility planning, and legal registration proof, is required, with strict adherence to the submission deadline and format. By channeling ODA directly into grassroots interventions, the program enhances local capacities, fosters socio-economic stability, and complements broader development efforts in Jordan.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>The Grant Assistance for Grassroots Human Security Projects (GGP) is part of Japan’s Official Development Assistance (ODA) framework, designed to support small-scale, community-focused initiatives that directly improve socio-economic conditions at the grassroots level in Jordan. Through this program, the Embassy of Japan seeks projects that deliver tangible benefits, from essential equipment procurement to community infrastructure renovations, supporting locally defined priorities and sustainable development outcomes. The funding logic emphasizes practical, operational impact and community ownership, prioritizing organizations with strong ties to their communities and demonstrated project delivery capacity. A comprehensive application, including financial audits, price quotations, feasibility planning, and legal registration proof, is required, with strict adherence to the submission deadline and format. By channeling ODA directly into grassroots interventions, the program enhances local capacities, fosters socio-economic stability, and complements broader development efforts in Jordan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/cross-cutting-intersectional-impact-bc1</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Misk Foundation</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>SAR 1,000,000 per winning track.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Saudi Arabia.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Community Development; Focus areas: technology‑driven solutions, health &amp; well‑being, environmental sustainability.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Saudi nonprofit organizations and social ventures focused on social or environmental innovation.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://hub.misk.org.sa/programs/community/challenge-for-change/ Misk Foundation</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>February 9, 2026.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Misk Foundation’s Challenge for Changeis a 7‑week hybrid acceleration and mentoring program designed to catalyze Saudi nonprofit and social ventures that address pressing social and environmental challenges. Across three thematic tracks, Technology, Health &amp; Well‑Being, and Environment, participants receive tailored bootcamps, one‑on‑one mentorship, and expert guidance to refine their impact strategies and scale meaningful solutions. The program culminates in a competitive pitch phase where winning teams in each track can secure SAR 1M in grant funding to implement their project ideas. This experiential learning journey equips changemakers with the practical skills, networks, and resources to turn innovative concepts into sustainable community impact.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Misk Foundation’s Challenge for Changeis a 7‑week hybrid acceleration and mentoring program designed to catalyze Saudi nonprofit and social ventures that address pressing social and environmental challenges. Across three thematic tracks, Technology, Health &amp; Well‑Being, and Environment, participants receive tailored bootcamps, one‑on‑one mentorship, and expert guidance to refine their impact strategies and scale meaningful solutions. The program culminates in a competitive pitch phase where winning teams in each track can secure SAR 1M in grant funding to implement their project ideas. This experiential learning journey equips changemakers with the practical skills, networks, and resources to turn innovative concepts into sustainable community impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/cross-cutting-intersectional-impact-b32</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Arab Fund for Arts and Culture (AFAC)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Grants range EUR €35,000- €65,000.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Algeria, Egypt, Jordan, Lebanon, Libya, Morocco, Palestine, Syria, Tunisia.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Arts and Culture; Focus areas: creative placemaking, interdisciplinary experimentation, cultural circulation.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Individuals and organizations from eligible countries working at the intersection of culture and social change.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.arabculturefund.org/Programs/74</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>November 21, 2025.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>AFAC’s new multi-year program,Ecologies of Culture, supports creative responses to today’s most interconnected global challenges, from gender inequality and climate change to digital transformation and social fragmentation. With funding for up to 58 projects across nine MENA countries, the program invites artists, cultural workers, researchers, technologists, journalists, and educators to co-design solutions that center imagination, local context, and interdisciplinary collaboration. Applicants may apply through three streams:Creative Placemaking(community-rooted cultural projects),Creative Labs(experimental cross-sector initiatives), andCreative Caravans(distribution and media-based work).</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>AFAC’s new multi-year program,Ecologies of Culture, supports creative responses to today’s most interconnected global challenges, from gender inequality and climate change to digital transformation and social fragmentation. With funding for up to 58 projects across nine MENA countries, the program invites artists, cultural workers, researchers, technologists, journalists, and educators to co-design solutions that center imagination, local context, and interdisciplinary collaboration. Applicants may apply through three streams:Creative Placemaking(community-rooted cultural projects),Creative Labs(experimental cross-sector initiatives), andCreative Caravans(distribution and media-based work).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="80" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/cross-cutting-intersectional-impact</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Prince Claus Fund</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>EUR €10,000 per participant plus covered travel, visa and accommodation.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Algeria; Angola; Benin; Botswana; Burkina Faso; Burundi; Cabo Verde; Cameroon; Central African Republic; Chad; Comores; Congo; Cote D'Ivoire; Democratic Republic of the Congo; Djibouti; Egypt; Equatorial Guinea; Eritrea; Eswatini; Ethiopia; Gabon; Gambia; Ghana; Guinea; Guinea-Bissau; Kenya; Lesotho; Liberia; Libya; Madagascar; Malawi; Mali; Mauritania; Mauritius; Morocco; Mozambique; Namibia; Niger; Nigeria; Rwanda; Saint Helena; Sao Tome and Principe; Senegal; Sierra Leone; Somalia; South Africa; South Sudan; Sudan; Tanzania; Tunisia; Togo; Uganda; Zambia; Zimbabwe.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Arts &amp; Culture; architecture; urbanism; cultural practice; urban culture practices.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Individual mid‑career artists or cultural practitioners (7–15 years) based in eligible African countries, with an artistic practice related to architecture, spatial design or public urban culture; must communicate in English; arts managers or researchers without an individual artistic practice are not eligible.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>https://princeclausfund.nl/awards-and-programmes/fellows-award/building-beyond/cycle-5-call-for-applications</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>August 13, 2025 (17:00 Amsterdam time).</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>The Prince Claus Fund’s Building Beyond Cycle 5 selects nine mid-career individual artists and cultural practitioners from eligible African countries for a nine‑month multidisciplinary fellowship rooted in spatial and urban practice. Each fellow receives €10,000 plus funded travel, visa, and accommodation, and benefits from mentorship by three Senior Fellows, peer collaboration, a Lab Week in person, and a collective cohort project. The programme engages practitioners with personal creative practices in architecture, design, and public space who have demonstrated 7‑15 years of professional experience.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>The Prince Claus Fund’s Building Beyond Cycle 5 selects nine mid-career individual artists and cultural practitioners from eligible African countries for a nine‑month multidisciplinary fellowship rooted in spatial and urban practice. Each fellow receives €10,000 plus funded travel, visa, and accommodation, and benefits from mentorship by three Senior Fellows, peer collaboration, a Lab Week in person, and a collective cohort project. The programme engages practitioners with personal creative practices in architecture, design, and public space who have demonstrated 7‑15 years of professional experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="80" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/cross-cutting-intersectional-impact</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Flat6Labs</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>SAR 500K in seed funding, and a potential SAR 2,400,000 in follow-on funding.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Saudi Arabia.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Multisector.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Anyone residing in country.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>https://flat6labs.com/program/riyadh-seed-program-page/</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>August 16, 2025.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Seeks to support the innovation of Saudi Arabian startups, enhance their entrepreneurial skills, and create a space for the Saudi youth to develop their startups and scale up their businesses in the MENA region. The Flat6Labs Riyadh Seed Program will support startups with high growth potential and will annually provide more than 20 Saudi startups with seed funding over the next three years.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Seeks to support the innovation of Saudi Arabian startups, enhance their entrepreneurial skills, and create a space for the Saudi youth to develop their startups and scale up their businesses in the MENA region. The Flat6Labs Riyadh Seed Program will support startups with high growth potential and will annually provide more than 20 Saudi startups with seed funding over the next three years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/multi-sector-sustainable-development-883</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Interreg Euro-MED Programme</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Co-financing €600,000-€3.1 million. Applicants must provide a minimum of 11% of the total project costs.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Mediterranean region; Algeria, Cyprus, Egypt, France, Greece, Israel, Italy, Jordan, Lebanon, Malta, Palestine, Portugal, Spain, Tunisia, Türkiye.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Climate and environment, job creation, inclusion, health.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Public and private bodies, as  well as international organizations. All applicant must be established in the participating countries and legally registered there since at least two years from the launching date of this call.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.interregnextmed.eu/apply-for-funding/second-call-for-proposals/</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>April 15, 2025.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Interreg NEXT MED is a program funded by the European Union (EU) that supports transnational cooperation through the financing of joint projects which aim at making the Mediterranean area more resilient to the shared challenges it faces. The Call for Green Transition Projects provides €83.7 million in European Union’s funding to tackle climate challenges across the Mediterranean region. Projects that aim to contribute to smart, sustainable, fair development for all across the Mediterranean basin across four program priorities, including research and innovation, climate, energy and water, education and healthcare, and governance.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Interreg NEXT MED is a program funded by the European Union (EU) that supports transnational cooperation through the financing of joint projects which aim at making the Mediterranean area more resilient to the shared challenges it faces. The Call for Green Transition Projects provides €83.7 million in European Union’s funding to tackle climate challenges across the Mediterranean region. Projects that aim to contribute to smart, sustainable, fair development for all across the Mediterranean basin across four program priorities, including research and innovation, climate, energy and water, education and healthcare, and governance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="80" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/multi-sector-sustainable-development</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Interreg Euro-MED Programme</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Co-financing €600,000-€3.1 million. Applicants must provide a minimum of 11% of the total project costs.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Mediterranean region; Algeria, Cyprus, Egypt, France, Greece, Israel, Italy, Jordan, Lebanon, Malta, Palestine, Portugal, Spain, Tunisia, Türkiye.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Climate and environment, job creation, inclusion, health.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Public and private bodies, as  well as international organizations. All applicant must be established in the participating countries and legally registered there since at least two years from the launching date of this call.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.interregnextmed.eu/apply-for-funding/second-call-for-proposals/</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>April 15, 2025.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Interreg NEXT MED is a program funded by the European Union (EU) that supports transnational cooperation through the financing of joint projects which aim at making the Mediterranean area more resilient to the shared challenges it faces. The Call for Green Transition Projects provides €83.7 million in European Union’s funding to tackle climate challenges across the Mediterranean region. Projects that aim to contribute to smart, sustainable, fair development for all across the Mediterranean basin across four program priorities, including research and innovation, climate, energy and water, education and healthcare, and governance.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Interreg NEXT MED is a program funded by the European Union (EU) that supports transnational cooperation through the financing of joint projects which aim at making the Mediterranean area more resilient to the shared challenges it faces. The Call for Green Transition Projects provides €83.7 million in European Union’s funding to tackle climate challenges across the Mediterranean region. Projects that aim to contribute to smart, sustainable, fair development for all across the Mediterranean basin across four program priorities, including research and innovation, climate, energy and water, education and healthcare, and governance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="80" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/innovation-research-and-smart-cities-727</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>BRICS STI Framework Programme</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Country-specific; e.g. €50,000 (South Africa), L.E. 10M (Egypt), R1M (approx.).</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Brazil, Russia, India, China, South Africa, Egypt.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Scientific Research; Focus areas: water treatment, energy storage, food tech, pharma, sustainability.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Universities, research institutions, SMMEs, and innovators legally registered in BRICS countries; must form consortia with at least two national partners.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>http://brics-sti.org/index.php?p=new/40/</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>December 3, 2025 (15:00 Moscow Time).</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>This multinational R&amp;D call supports collaborative innovation among BRICS nations, targeting real-world solutions to shared societal challenges. Eligible institutions must partner across at least two BRICS countries and co-design projects that deliver scalable technologies in areas such as water sustainability, clean energy, medical innovation, and digital infrastructure. Proposals must reflect a clear path to impact—aligned with TRL 5–7—and be grounded in complementary expertise across the consortium. Funding is issued nationally, with each country applying its own regulations, instruments, and disbursement timelines.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>This multinational R&amp;D call supports collaborative innovation among BRICS nations, targeting real-world solutions to shared societal challenges. Eligible institutions must partner across at least two BRICS countries and co-design projects that deliver scalable technologies in areas such as water sustainability, clean energy, medical innovation, and digital infrastructure. Proposals must reflect a clear path to impact—aligned with TRL 5–7—and be grounded in complementary expertise across the consortium. Funding is issued nationally, with each country applying its own regulations, instruments, and disbursement timelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="80" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>https://impactfunding.substack.com/p/innovation-research-and-smart-cities-215</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Driving Urban Transitions (DUT) Partnership</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>€1–2 million per project (approx.); Total pool: €44 million.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Austria, Belgium, Croatia, Czech Republic, Denmark, Estonia, Finland, France, Germany, Italy, Republic of Korea, Latvia, Lithuania, Malta, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden, Switzerland, The Netherlands, Tunisia, Türkiye.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Urban Development; Focus areas: circular urban economies, 15-minute city, energy-positive districts, integrated planning.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Transnational consortia with at least 3 partners from 3 of the participating countries; organizations must check national annexes for eligibility.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>https://dutpartnership.eu/calls/dut-call-2025#before-you-apply-303</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>November 17, 2025 .</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>This Horizon Europe-aligned transnational call funds R&amp;I projects focused on accelerating urban sustainability transitions. Applicants must form a consortium of at least three entities from three of the 26 participating countries. The call prioritizes solutions aligned with three interconnected thematic pillars: Positive Energy Districts, the 15-minute City, and Circular Urban Economies. Funding is provided through national/regional agencies- each with their own eligibility and budget frameworks.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>This Horizon Europe-aligned transnational call funds R&amp;I projects focused on accelerating urban sustainability transitions. Applicants must form a consortium of at least three entities from three of the 26 participating countries. The call prioritizes solutions aligned with three interconnected thematic pillars: Positive Energy Districts, the 15-minute City, and Circular Urban Economies. Funding is provided through national/regional agencies- each with their own eligibility and budget frameworks.</t>
         </is>
       </c>
     </row>

</xml_diff>